<commit_message>
added wbs columns to conf report and changed historical ref error text
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/ConfidenceReport.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/ConfidenceReport.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673B041D-C873-4DB0-9B37-67F895E96C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FDB4411-FB60-4885-AB86-FBC396FE2EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3870" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-8780" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Confidence Report" sheetId="1" r:id="rId1"/>
     <sheet name="Options Lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Confidence Report'!$A$2:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Confidence Report'!$A$2:$H$2</definedName>
     <definedName name="ContractTypes">'Options Lists'!$A$2</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>ContractTypes</t>
   </si>
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t>Confidence Error Messages</t>
+  </si>
+  <si>
+    <t>WBS #</t>
+  </si>
+  <si>
+    <t>WBS Title</t>
   </si>
 </sst>
 </file>
@@ -439,39 +445,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="18.5703125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="56.28515625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="58.28515625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="16.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="31" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="30.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="40.5546875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="18.5546875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="56.33203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="58.33203125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:7" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:7" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A2:E2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:H2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -484,12 +498,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -505,15 +519,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -616,6 +621,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
@@ -630,14 +644,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CFE6607-7799-4DB1-BBAD-BE0483ACB310}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -656,6 +662,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
added tool tips and urls
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/ConfidenceReport.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/ConfidenceReport.xlsx
@@ -3,16 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FDB4411-FB60-4885-AB86-FBC396FE2EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F57226-49A0-415F-904F-C9261AB7C598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-8780" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Confidence Report" sheetId="1" r:id="rId1"/>
     <sheet name="Options Lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Confidence Report'!$A$2:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Confidence Report'!$A$2:$J$2</definedName>
     <definedName name="ContractTypes">'Options Lists'!$A$2</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>ContractTypes</t>
   </si>
@@ -44,6 +44,12 @@
   </si>
   <si>
     <t>WBS Title</t>
+  </si>
+  <si>
+    <t>BOE URL</t>
+  </si>
+  <si>
+    <t>Task URL</t>
   </si>
 </sst>
 </file>
@@ -445,22 +451,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="1" customWidth="1"/>
-    <col min="3" max="3" width="31.109375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="30.6640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="40.5546875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="18.5546875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="56.33203125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="58.33203125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="1"/>
+    <col min="3" max="4" width="31.109375" style="4" customWidth="1"/>
+    <col min="5" max="6" width="30.6640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="40.5546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="18.5546875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="56.33203125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="58.33203125" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="1:7" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" s="2" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -471,21 +477,27 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:9" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A2:H2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:J2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -519,6 +531,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -621,29 +655,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CFE6607-7799-4DB1-BBAD-BE0483ACB310}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -660,29 +697,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDA7760-8C18-4744-80BE-EC14AF3979C1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E141511F-2C2D-45F4-A120-F9C297666AB6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>